<commit_message>
Park note links: remove the link button and shortcut
</commit_message>
<xml_diff>
--- a/examples/Lanetrace-Template.xlsx
+++ b/examples/Lanetrace-Template.xlsx
@@ -303,7 +303,7 @@
     <t xml:space="preserve">Text with basic Markdown</t>
   </si>
   <si>
-    <t xml:space="preserve">Detail for the tooltip and item panel. Supports **bold**, *italic*, - bullets and [links](https://...).</t>
+    <t xml:space="preserve">Detail for the tooltip and item panel. Supports **bold**, *italic*, # headings, - bullets and 1. numbered lists.</t>
   </si>
   <si>
     <t xml:space="preserve">**Scope:** login, profile</t>
@@ -336,7 +336,7 @@
     <t xml:space="preserve">Whole number 1 to 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Moves a milestone, event or decision out of its swimlane into that row of the strip above the timescale. Blank keeps it in its swimlane.</t>
+    <t xml:space="preserve">Moves a milestone, event or decision out of its swimlane into that row of the strip above the timescale, with the Lanetrace setting Milestones: As set per item (the default). Blank keeps it in its swimlane.</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
@@ -1158,7 +1158,7 @@
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Owner" prompt="Person or team responsible. Shows in the tooltip and the status update." sqref="H2:H5000"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Depends on" prompt="Row IDs of items that must finish before this one starts, separated by commas, like 3, 5. Leave blank if none." sqref="I2:I5000"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Notes" prompt="Detail for the tooltip and item panel. Supports **bold**, *italic*, - bullets and [text](https://link)." sqref="J2:J5000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Notes" prompt="Detail for the tooltip and item panel. Supports **bold**, *italic*, # headings, - bullets and 1. numbered lists." sqref="J2:J5000"/>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Item Type" error="Pick a value from the list." showInputMessage="1" promptTitle="Item Type" prompt="Blank lets Lanetrace decide: no start date or a same-day start and end = Milestone, 92 days or less = Task, longer = Phase." sqref="K2:K5000">
       <formula1>"Task,Phase,Milestone,Event,Decision"</formula1>
     </dataValidation>
@@ -1547,7 +1547,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="35" ht="49" customHeight="1">
+    <row r="35" ht="63" customHeight="1">
       <c r="A35" s="12" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Template instructions: headers ignore capitals; CSV loads the same way
</commit_message>
<xml_diff>
--- a/examples/Lanetrace-Template.xlsx
+++ b/examples/Lanetrace-Template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="192">
   <si>
     <t xml:space="preserve">Row ID</t>
   </si>
@@ -444,7 +444,13 @@
     <t xml:space="preserve">Headers</t>
   </si>
   <si>
-    <t xml:space="preserve">Lanetrace matches columns by exact header text. A renamed header is ignored, and the load message names the missing required columns. Extra columns of your own are fine.</t>
+    <t xml:space="preserve">Lanetrace matches columns by header text; capitals do not matter. A renamed header is ignored, and the load message names the missing required columns. Extra columns of your own are fine.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A CSV file with these same headers loads the same way, for example a CSV UTF-8 saved from Excel. Commas, semicolons or tabs all work.</t>
   </si>
   <si>
     <t xml:space="preserve">List the Row IDs of items that must finish before this one starts. Lanetrace flags an item that starts before a predecessor finishes, an ID that matches no row, and a chain that loops back on itself. It never moves your dates.</t>
@@ -585,7 +591,7 @@
     <t xml:space="preserve">Remove one Row ID from the loop.</t>
   </si>
   <si>
-    <t xml:space="preserve">Template for Lanetrace v4.12.0. Created 2026-10-15. Sample dates start in the current month.</t>
+    <t xml:space="preserve">Template for Lanetrace v4.12.0. Created 2026-10-16. Sample dates start in the current month.</t>
   </si>
 </sst>
 </file>
@@ -1194,7 +1200,7 @@
     <tabColor rgb="FF14181F"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1796,10 +1802,10 @@
     </row>
     <row r="56" ht="35" customHeight="1">
       <c r="A56" s="12" t="s">
-        <v>8</v>
+        <v>143</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C56" s="11"/>
       <c r="D56" s="11"/>
@@ -1807,18 +1813,18 @@
     </row>
     <row r="57" ht="35" customHeight="1">
       <c r="A57" s="12" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C57" s="11"/>
       <c r="D57" s="11"/>
       <c r="E57" s="11"/>
     </row>
-    <row r="58" ht="21" customHeight="1">
+    <row r="58" ht="35" customHeight="1">
       <c r="A58" s="12" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>146</v>
@@ -1827,34 +1833,34 @@
       <c r="D58" s="11"/>
       <c r="E58" s="11"/>
     </row>
-    <row r="59" ht="16" customHeight="1"/>
-    <row r="60" ht="24" customHeight="1">
-      <c r="A60" s="9" t="s">
+    <row r="59" ht="21" customHeight="1">
+      <c r="A59" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-    </row>
-    <row r="61" ht="6" customHeight="1"/>
-    <row r="62" ht="21" customHeight="1">
-      <c r="A62" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B62" s="11" t="s">
+      <c r="B59" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="C62" s="11"/>
-      <c r="D62" s="11"/>
-      <c r="E62" s="11"/>
-    </row>
+      <c r="C59" s="11"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+    </row>
+    <row r="60" ht="16" customHeight="1"/>
+    <row r="61" ht="24" customHeight="1">
+      <c r="A61" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+    </row>
+    <row r="62" ht="6" customHeight="1"/>
     <row r="63" ht="21" customHeight="1">
       <c r="A63" s="12" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C63" s="11"/>
       <c r="D63" s="11"/>
@@ -1862,7 +1868,7 @@
     </row>
     <row r="64" ht="21" customHeight="1">
       <c r="A64" s="12" t="s">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>151</v>
@@ -1871,7 +1877,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="11"/>
     </row>
-    <row r="65" ht="35" customHeight="1">
+    <row r="65" ht="21" customHeight="1">
       <c r="A65" s="12" t="s">
         <v>152</v>
       </c>
@@ -1893,7 +1899,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="11"/>
     </row>
-    <row r="67" ht="21" customHeight="1">
+    <row r="67" ht="35" customHeight="1">
       <c r="A67" s="12" t="s">
         <v>156</v>
       </c>
@@ -1904,155 +1910,166 @@
       <c r="D67" s="11"/>
       <c r="E67" s="11"/>
     </row>
-    <row r="68" ht="16" customHeight="1"/>
-    <row r="69" ht="24" customHeight="1">
-      <c r="A69" s="9" t="s">
+    <row r="68" ht="21" customHeight="1">
+      <c r="A68" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9"/>
-    </row>
-    <row r="70" ht="6" customHeight="1"/>
-    <row r="71" ht="21" customHeight="1">
-      <c r="A71" s="10" t="s">
+      <c r="B68" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="B71" s="10"/>
-      <c r="C71" s="10" t="s">
+      <c r="C68" s="11"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="11"/>
+    </row>
+    <row r="69" ht="16" customHeight="1"/>
+    <row r="70" ht="24" customHeight="1">
+      <c r="A70" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="D71" s="10" t="s">
+      <c r="B70" s="9"/>
+      <c r="C70" s="9"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="9"/>
+    </row>
+    <row r="71" ht="6" customHeight="1"/>
+    <row r="72" ht="21" customHeight="1">
+      <c r="A72" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="E71" s="10"/>
-    </row>
-    <row r="72" ht="21" customHeight="1">
-      <c r="A72" s="12" t="s">
+      <c r="B72" s="10"/>
+      <c r="C72" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B72" s="12"/>
-      <c r="C72" s="11" t="s">
+      <c r="D72" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="D72" s="11" t="s">
+      <c r="E72" s="10"/>
+    </row>
+    <row r="73" ht="21" customHeight="1">
+      <c r="A73" s="12" t="s">
         <v>164</v>
-      </c>
-      <c r="E72" s="11"/>
-    </row>
-    <row r="73" ht="35" customHeight="1">
-      <c r="A73" s="12" t="s">
-        <v>165</v>
       </c>
       <c r="B73" s="12"/>
       <c r="C73" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="D73" s="11" t="s">
         <v>166</v>
-      </c>
-      <c r="D73" s="11" t="s">
-        <v>167</v>
       </c>
       <c r="E73" s="11"/>
     </row>
     <row r="74" ht="35" customHeight="1">
       <c r="A74" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B74" s="12"/>
       <c r="C74" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D74" s="11" t="s">
         <v>169</v>
-      </c>
-      <c r="D74" s="11" t="s">
-        <v>170</v>
       </c>
       <c r="E74" s="11"/>
     </row>
     <row r="75" ht="35" customHeight="1">
       <c r="A75" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B75" s="12"/>
       <c r="C75" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D75" s="11" t="s">
         <v>172</v>
-      </c>
-      <c r="D75" s="11" t="s">
-        <v>173</v>
       </c>
       <c r="E75" s="11"/>
     </row>
     <row r="76" ht="35" customHeight="1">
       <c r="A76" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B76" s="12"/>
       <c r="C76" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="D76" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="D76" s="11" t="s">
+      <c r="E76" s="11"/>
+    </row>
+    <row r="77" ht="35" customHeight="1">
+      <c r="A77" s="12" t="s">
         <v>176</v>
-      </c>
-      <c r="E76" s="11"/>
-    </row>
-    <row r="77" ht="21" customHeight="1">
-      <c r="A77" s="12" t="s">
-        <v>177</v>
       </c>
       <c r="B77" s="12"/>
       <c r="C77" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="D77" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="D77" s="11" t="s">
+      <c r="E77" s="11"/>
+    </row>
+    <row r="78" ht="21" customHeight="1">
+      <c r="A78" s="12" t="s">
         <v>179</v>
-      </c>
-      <c r="E77" s="11"/>
-    </row>
-    <row r="78" ht="49" customHeight="1">
-      <c r="A78" s="12" t="s">
-        <v>180</v>
       </c>
       <c r="B78" s="12"/>
       <c r="C78" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="D78" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="D78" s="11" t="s">
+      <c r="E78" s="11"/>
+    </row>
+    <row r="79" ht="49" customHeight="1">
+      <c r="A79" s="12" t="s">
         <v>182</v>
-      </c>
-      <c r="E78" s="11"/>
-    </row>
-    <row r="79" ht="35" customHeight="1">
-      <c r="A79" s="12" t="s">
-        <v>183</v>
       </c>
       <c r="B79" s="12"/>
       <c r="C79" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D79" s="11" t="s">
         <v>184</v>
-      </c>
-      <c r="D79" s="11" t="s">
-        <v>185</v>
       </c>
       <c r="E79" s="11"/>
     </row>
     <row r="80" ht="35" customHeight="1">
       <c r="A80" s="12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B80" s="12"/>
       <c r="C80" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="D80" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="D80" s="11" t="s">
+      <c r="E80" s="11"/>
+    </row>
+    <row r="81" ht="35" customHeight="1">
+      <c r="A81" s="12" t="s">
         <v>188</v>
       </c>
-      <c r="E80" s="11"/>
-    </row>
-    <row r="81" ht="18" customHeight="1"/>
-    <row r="82" ht="16" customHeight="1">
-      <c r="A82" s="15" t="s">
+      <c r="B81" s="12"/>
+      <c r="C81" s="11" t="s">
         <v>189</v>
       </c>
+      <c r="D81" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="E81" s="11"/>
+    </row>
+    <row r="82" ht="18" customHeight="1"/>
+    <row r="83" ht="16" customHeight="1">
+      <c r="A83" s="15" t="s">
+        <v>191</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="41">
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="B10:E10"/>
@@ -2067,14 +2084,13 @@
     <mergeCell ref="B56:E56"/>
     <mergeCell ref="B57:E57"/>
     <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="B59:E59"/>
     <mergeCell ref="B63:E63"/>
     <mergeCell ref="B64:E64"/>
     <mergeCell ref="B65:E65"/>
     <mergeCell ref="B66:E66"/>
     <mergeCell ref="B67:E67"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="B68:E68"/>
     <mergeCell ref="A72:B72"/>
     <mergeCell ref="D72:E72"/>
     <mergeCell ref="A73:B73"/>
@@ -2093,6 +2109,8 @@
     <mergeCell ref="D79:E79"/>
     <mergeCell ref="A80:B80"/>
     <mergeCell ref="D80:E80"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="D81:E81"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Lanetrace 4.16.0: Description and Updates fields, Milestones view, Insert above/below keeps its place
- Description under the title in the item form and tooltip, with Data view, Excel and CSV columns
- Updates: a running log; each entry is saved with its date and time, newest first
- Data view: Milestones layout (milestones, events and decisions by date); Start and End read MM/DD/YYYY
- Notes toolbar Expand button
- Insert row above/below puts the row next to the selected row, with a saved row order
- A new row with no dates no longer stops the timeline from drawing
</commit_message>
<xml_diff>
--- a/examples/Lanetrace-Template.xlsx
+++ b/examples/Lanetrace-Template.xlsx
@@ -9,14 +9,14 @@
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TimelineExcel!$A$1:$R$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TimelineExcel!$A$1:$U$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">TimelineExcel!$1:$1</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205">
   <si>
     <t xml:space="preserve">Row ID</t>
   </si>
@@ -30,6 +30,9 @@
     <t xml:space="preserve">Milestone/Task Title</t>
   </si>
   <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
     <t xml:space="preserve">Start date</t>
   </si>
   <si>
@@ -48,6 +51,9 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
+    <t xml:space="preserve">Updates</t>
+  </si>
+  <si>
     <t xml:space="preserve">Item Type</t>
   </si>
   <si>
@@ -72,12 +78,18 @@
     <t xml:space="preserve">Title Color</t>
   </si>
   <si>
+    <t xml:space="preserve">Health</t>
+  </si>
+  <si>
     <t xml:space="preserve">Product</t>
   </si>
   <si>
     <t xml:space="preserve">Discovery and requirements</t>
   </si>
   <si>
+    <t xml:space="preserve">Customer interviews and a journey map, ending in the requirements the build starts from</t>
+  </si>
+  <si>
     <t xml:space="preserve">Product team</t>
   </si>
   <si>
@@ -111,6 +123,12 @@
     <t xml:space="preserve">Item Type left blank: Lanetrace reads the dates and draws a Phase.</t>
   </si>
   <si>
+    <t xml:space="preserve">[10/03/2026 9:30 AM] Auth service is two weeks behind, so Health is At Risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At Risk</t>
+  </si>
+  <si>
     <t xml:space="preserve">Frontend</t>
   </si>
   <si>
@@ -261,6 +279,15 @@
     <t xml:space="preserve">The label on the timeline.</t>
   </si>
   <si>
+    <t xml:space="preserve">Text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What the item covers: scope, deliverables, definition of done. Shows under the title in the tooltip and item form.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configure surveys for 22 service lines</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date</t>
   </si>
   <si>
@@ -285,9 +312,6 @@
     <t xml:space="preserve">40</t>
   </si>
   <si>
-    <t xml:space="preserve">Text</t>
-  </si>
-  <si>
     <t xml:space="preserve">Person or team responsible. Shows in the tooltip and the status update.</t>
   </si>
   <si>
@@ -309,6 +333,15 @@
     <t xml:space="preserve">**Scope:** login, profile</t>
   </si>
   <si>
+    <t xml:space="preserve">Dated entries, newest first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running status log. Lanetrace adds each new update to the top with its date and time. One entry per line, starting with the stamp in brackets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[10/29/2026 2:05 PM] Vendor confirmed the SFTP account</t>
+  </si>
+  <si>
     <t xml:space="preserve">Task, Phase, Milestone, Event, Decision</t>
   </si>
   <si>
@@ -360,6 +393,12 @@
     <t xml:space="preserve">Auto picks white or dark text for contrast. Set it only to override.</t>
   </si>
   <si>
+    <t xml:space="preserve">On Track, At Risk, Off Track</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your read on the item. Blank is Auto: Lanetrace works it out from the dates and % complete. Green, Amber and Red also work.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Item types</t>
   </si>
   <si>
@@ -591,7 +630,7 @@
     <t xml:space="preserve">Remove one Row ID from the loop.</t>
   </si>
   <si>
-    <t xml:space="preserve">Template for Lanetrace v4.12.0. Created 2026-10-16. Sample dates start in the current month.</t>
+    <t xml:space="preserve">Template for Lanetrace v4.16.0. Created 2026-10-29. Sample dates start in the current month.</t>
   </si>
 </sst>
 </file>
@@ -766,27 +805,30 @@
     <tabColor rgb="FF1E4FD8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="11" style="5" customWidth="1"/>
     <col min="2" max="2" width="20" style="3" customWidth="1"/>
     <col min="3" max="3" width="18" style="3" customWidth="1"/>
     <col min="4" max="4" width="40" style="4" customWidth="1"/>
-    <col min="5" max="5" width="15" style="6" customWidth="1"/>
+    <col min="5" max="5" width="40" style="4" customWidth="1"/>
     <col min="6" max="6" width="15" style="6" customWidth="1"/>
-    <col min="7" max="7" width="15" style="5" customWidth="1"/>
-    <col min="8" max="8" width="18" style="3" customWidth="1"/>
-    <col min="9" max="9" width="14" style="5" customWidth="1"/>
-    <col min="10" max="10" width="46" style="4" customWidth="1"/>
-    <col min="11" max="11" width="14" style="3" customWidth="1"/>
-    <col min="12" max="12" width="17" style="3" customWidth="1"/>
-    <col min="13" max="13" width="20" style="3" customWidth="1"/>
-    <col min="14" max="14" width="13" style="3" customWidth="1"/>
-    <col min="15" max="15" width="18" style="5" customWidth="1"/>
-    <col min="16" max="16" width="11" style="3" customWidth="1"/>
+    <col min="7" max="7" width="15" style="6" customWidth="1"/>
+    <col min="8" max="8" width="15" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14" style="5" customWidth="1"/>
+    <col min="11" max="11" width="46" style="4" customWidth="1"/>
+    <col min="12" max="12" width="46" style="4" customWidth="1"/>
+    <col min="13" max="13" width="14" style="3" customWidth="1"/>
+    <col min="14" max="14" width="17" style="3" customWidth="1"/>
+    <col min="15" max="15" width="20" style="3" customWidth="1"/>
+    <col min="16" max="16" width="13" style="3" customWidth="1"/>
     <col min="17" max="17" width="18" style="5" customWidth="1"/>
-    <col min="18" max="18" width="14" style="3" customWidth="1"/>
+    <col min="18" max="18" width="11" style="3" customWidth="1"/>
+    <col min="19" max="19" width="18" style="5" customWidth="1"/>
+    <col min="20" max="20" width="14" style="3" customWidth="1"/>
+    <col min="21" max="21" width="13" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -805,10 +847,10 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
@@ -844,349 +886,393 @@
       <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="5">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="6">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="6">
         <v>46296</v>
       </c>
-      <c r="F2" s="6">
+      <c r="G2" s="6">
         <v>46356</v>
       </c>
-      <c r="G2" s="5">
+      <c r="H2" s="5">
         <v>100</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" s="5"/>
-      <c r="J2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="5"/>
+      <c r="K2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" s="4"/>
+      <c r="M2" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="N2" s="3"/>
-      <c r="O2" s="5"/>
+      <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="3"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
     </row>
     <row r="3">
       <c r="A3" s="5">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6">
+        <v>27</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6">
         <v>46356</v>
       </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" s="5"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="5"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="3" t="s">
+        <v>29</v>
+      </c>
       <c r="N3" s="3"/>
-      <c r="O3" s="5"/>
+      <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="3"/>
+      <c r="S3" s="5"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="6">
+        <v>32</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="6">
         <v>46327</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>46446</v>
       </c>
-      <c r="G4" s="5">
+      <c r="H4" s="5">
         <v>40</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I4" s="5"/>
-      <c r="J4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="5"/>
+      <c r="K4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
-      <c r="O4" s="5"/>
+      <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="5"/>
       <c r="R4" s="3"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="6">
+        <v>38</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="6">
         <v>46357</v>
       </c>
-      <c r="F5" s="6">
+      <c r="G5" s="6">
         <v>46446</v>
       </c>
-      <c r="G5" s="5">
+      <c r="H5" s="5">
         <v>15</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5" s="4"/>
-      <c r="K5" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="M5" s="3"/>
+      <c r="I5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="N5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="O5" s="5"/>
-      <c r="P5" s="3"/>
+        <v>42</v>
+      </c>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3" t="s">
+        <v>43</v>
+      </c>
       <c r="Q5" s="5"/>
       <c r="R5" s="3"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
     </row>
     <row r="6">
       <c r="A6" s="5">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6">
+        <v>44</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6">
         <v>46341</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" s="5"/>
-      <c r="J6" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6" s="5"/>
+      <c r="K6" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="L6" s="4"/>
+      <c r="M6" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="N6" s="3"/>
-      <c r="O6" s="5"/>
+      <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="5"/>
       <c r="R6" s="3"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="3"/>
+      <c r="U6" s="3"/>
     </row>
     <row r="7">
       <c r="A7" s="5">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6">
+        <v>49</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6">
         <v>46456</v>
       </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I7" s="5"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="5"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="O7" s="3"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="5"/>
       <c r="R7" s="3"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
     </row>
     <row r="8">
       <c r="A8" s="5">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6">
+        <v>53</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6">
         <v>46477</v>
       </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J8" s="4"/>
-      <c r="K8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L8" s="3"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
       <c r="M8" s="3" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="N8" s="3"/>
-      <c r="O8" s="5"/>
+      <c r="O8" s="3" t="s">
+        <v>56</v>
+      </c>
       <c r="P8" s="3"/>
-      <c r="Q8" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="Q8" s="5"/>
       <c r="R8" s="3"/>
+      <c r="S8" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="6">
+        <v>46478</v>
+      </c>
+      <c r="G9" s="6">
+        <v>46538</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E9" s="6">
-        <v>46478</v>
-      </c>
-      <c r="F9" s="6">
-        <v>46538</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
+      <c r="J9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="L9" s="4"/>
+      <c r="M9" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="N9" s="3"/>
-      <c r="O9" s="5"/>
-      <c r="P9" s="3" t="s">
-        <v>55</v>
-      </c>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
       <c r="Q9" s="5"/>
-      <c r="R9" s="3"/>
+      <c r="R9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="S9" s="5"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R9"/>
-  <dataValidations count="18">
+  <autoFilter ref="A1:U9"/>
+  <dataValidations count="21">
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Row ID" prompt="A unique number or code for this row. Keep it the same between versions of the file." sqref="A2:A5000"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Swimlane" prompt="Top-level group, like a team or workstream. Each new name becomes a swimlane." sqref="B2:B5000"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Sub-swimlane" prompt="Optional second level inside a swimlane. Leave blank to keep the item in the main swimlane row." sqref="C2:C5000"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Milestone/Task Title" prompt="The label shown on the timeline. Under about 60 characters fits best." sqref="D2:D5000"/>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" errorTitle="Start date" error="Enter a date, like 2026-03-31. Text like TBD cannot be placed on the timeline." showInputMessage="1" promptTitle="Start date" prompt="First day of a task or phase. Leave blank for a milestone, event or decision." sqref="E2:E5000">
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="What the item covers: scope, deliverables, definition of done. Shows under the title in the tooltip and item form." sqref="E2:E5000"/>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" errorTitle="Start date" error="Enter a date, like 2026-03-31. Text like TBD cannot be placed on the timeline." showInputMessage="1" promptTitle="Start date" prompt="First day of a task or phase. Leave blank for a milestone, event or decision." sqref="F2:F5000">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" errorTitle="End date" error="Enter a date, like 2026-03-31. Text like TBD cannot be placed on the timeline." showInputMessage="1" promptTitle="End date" prompt="Last day of a task or phase, or the date of a milestone, event or decision." sqref="F2:F5000">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" errorTitle="End date" error="Enter a date, like 2026-03-31. Text like TBD cannot be placed on the timeline." showInputMessage="1" promptTitle="End date" prompt="Last day of a task or phase, or the date of a milestone, event or decision." sqref="G2:G5000">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="% Complete" error="Enter a whole number from 0 to 100, without a % sign." showInputMessage="1" promptTitle="% Complete" prompt="Whole number from 0 to 100, without a % sign. Blank counts as 0." sqref="G2:G5000">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="% Complete" error="Enter a whole number from 0 to 100, without a % sign." showInputMessage="1" promptTitle="% Complete" prompt="Whole number from 0 to 100, without a % sign. Blank counts as 0." sqref="H2:H5000">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Owner" prompt="Person or team responsible. Shows in the tooltip and the status update." sqref="H2:H5000"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Depends on" prompt="Row IDs of items that must finish before this one starts, separated by commas, like 3, 5. Leave blank if none." sqref="I2:I5000"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Notes" prompt="Detail for the tooltip and item panel. Supports **bold**, *italic*, # headings, - bullets and 1. numbered lists." sqref="J2:J5000"/>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Item Type" error="Pick a value from the list." showInputMessage="1" promptTitle="Item Type" prompt="Blank lets Lanetrace decide: no start date or a same-day start and end = Milestone, 92 days or less = Task, longer = Phase." sqref="K2:K5000">
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Owner" prompt="Person or team responsible. Shows in the tooltip and the status update." sqref="I2:I5000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Depends on" prompt="Row IDs of items that must finish before this one starts, separated by commas, like 3, 5. Leave blank if none." sqref="J2:J5000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Notes" prompt="Detail for the tooltip and item panel. Supports **bold**, *italic*, # headings, - bullets and 1. numbered lists." sqref="K2:K5000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Updates" prompt="Running status log, newest first. Each entry starts with its date and time in brackets, like [10/29/2026 2:05 PM]." sqref="L2:L5000"/>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Item Type" error="Pick a value from the list." showInputMessage="1" promptTitle="Item Type" prompt="Blank lets Lanetrace decide: no start date or a same-day start and end = Milestone, 92 days or less = Task, longer = Phase." sqref="M2:M5000">
       <formula1>"Task,Phase,Milestone,Event,Decision"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Label Position" error="Pick a value from the list." showInputMessage="1" promptTitle="Label Position" prompt="Where the title sits. Auto puts it inside the bar when it fits, otherwise beside it." sqref="L2:L5000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Label Position" error="Pick a value from the list." showInputMessage="1" promptTitle="Label Position" prompt="Where the title sits. Auto puts it inside the bar when it fits, otherwise beside it." sqref="N2:N5000">
       <formula1>"Auto,Above,Below,Left,Right,Inside"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Milestone Shape" error="Pick a value from the list." showInputMessage="1" promptTitle="Milestone Shape" prompt="Marker shape for a milestone, event or decision. Leave blank for the type default." sqref="M2:M5000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Milestone Shape" error="Pick a value from the list." showInputMessage="1" promptTitle="Milestone Shape" prompt="Marker shape for a milestone, event or decision. Leave blank for the type default." sqref="O2:O5000">
       <formula1>"diamond,diamond-tall,circle,triangle-right,triangle-down,triangle-down-large,star,flag"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Bar Style" error="Pick a value from the list." showInputMessage="1" promptTitle="Bar Style" prompt="Bar ends for a task or phase. Leave blank: tasks get Chevron, phases get Pill." sqref="N2:N5000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Bar Style" error="Pick a value from the list." showInputMessage="1" promptTitle="Bar Style" prompt="Bar ends for a task or phase. Leave blank: tasks get Chevron, phases get Pill." sqref="P2:P5000">
       <formula1>"Flat,Chevron,Pill"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Milestone Row" error="Enter a whole number from 1 to 6." showInputMessage="1" promptTitle="Milestone Row" prompt="Moves this milestone, event or decision into row 1 to 6 of the strip above the timescale. Blank keeps it in its swimlane." sqref="O2:O5000">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Milestone Row" error="Enter a whole number from 1 to 6." showInputMessage="1" promptTitle="Milestone Row" prompt="Moves this milestone, event or decision into row 1 to 6 of the strip above the timescale. Blank keeps it in its swimlane." sqref="Q2:Q5000">
       <formula1>1</formula1>
       <formula2>6</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Shown" error="Pick a value from the list." showInputMessage="1" promptTitle="Shown" prompt="No hides the item without deleting it. Blank or Yes shows it." sqref="P2:P5000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Shown" error="Pick a value from the list." showInputMessage="1" promptTitle="Shown" prompt="No hides the item without deleting it. Blank or Yes shows it." sqref="R2:R5000">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Color Category" prompt="A hex color like #E2A32D. Overrides the swimlane color for this item." sqref="Q2:Q5000"/>
-    <dataValidation type="list" allowBlank="1" errorStyle="information" showErrorMessage="1" errorTitle="Title Color" error="Not one of the listed values. Lanetrace also accepts a hex color like #1A1F2B." showInputMessage="1" promptTitle="Title Color" prompt="Auto picks white or dark text for contrast. Choose White or Dark, or type a hex color, to override." sqref="R2:R5000">
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Color Category" prompt="A hex color like #E2A32D. Overrides the swimlane color for this item." sqref="S2:S5000"/>
+    <dataValidation type="list" allowBlank="1" errorStyle="information" showErrorMessage="1" errorTitle="Title Color" error="Not one of the listed values. Lanetrace also accepts a hex color like #1A1F2B." showInputMessage="1" promptTitle="Title Color" prompt="Auto picks white or dark text for contrast. Choose White or Dark, or type a hex color, to override." sqref="T2:T5000">
       <formula1>"Auto,White,Dark"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" errorStyle="information" showErrorMessage="1" errorTitle="Health" error="Not one of the listed values. Lanetrace also reads Green, Amber, Yellow and Red, and keeps other text as typed." showInputMessage="1" promptTitle="Health" prompt="On Track, At Risk or Off Track. Leave blank for Auto, which Lanetrace works out from the dates and % complete." sqref="U2:U5000">
+      <formula1>"On Track,At Risk,Off Track"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -1200,7 +1286,7 @@
     <tabColor rgb="FF14181F"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1212,18 +1298,18 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -1236,7 +1322,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" ht="4" customHeight="1"/>
@@ -1245,7 +1331,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" ht="4" customHeight="1"/>
@@ -1254,7 +1340,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" ht="4" customHeight="1"/>
@@ -1263,7 +1349,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" ht="4" customHeight="1"/>
@@ -1272,13 +1358,13 @@
         <v>5</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1"/>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -1288,10 +1374,10 @@
     <row r="17" ht="6" customHeight="1"/>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="17" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
@@ -1300,19 +1386,19 @@
     <row r="19" ht="6" customHeight="1"/>
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="10" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" ht="35" customHeight="1">
@@ -1320,16 +1406,16 @@
         <v>0</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" ht="35" customHeight="1">
@@ -1337,16 +1423,16 @@
         <v>1</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" ht="35" customHeight="1">
@@ -1354,16 +1440,16 @@
         <v>2</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" ht="21" customHeight="1">
@@ -1371,16 +1457,16 @@
         <v>3</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" ht="35" customHeight="1">
@@ -1388,67 +1474,67 @@
         <v>4</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" ht="35" customHeight="1">
       <c r="A26" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B26" s="17" t="s">
-        <v>68</v>
+      <c r="B26" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="27" ht="21" customHeight="1">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" ht="35" customHeight="1">
       <c r="A27" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="11" t="s">
-        <v>77</v>
+      <c r="B27" s="17" t="s">
+        <v>74</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="28" ht="35" customHeight="1">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28" ht="21" customHeight="1">
       <c r="A28" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>29</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29" ht="35" customHeight="1">
@@ -1456,16 +1542,16 @@
         <v>8</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>93</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" ht="35" customHeight="1">
@@ -1473,16 +1559,16 @@
         <v>9</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" ht="35" customHeight="1">
@@ -1490,50 +1576,50 @@
         <v>10</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" ht="35" customHeight="1">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="32" ht="49" customHeight="1">
       <c r="A32" s="12" t="s">
         <v>11</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="33" ht="63" customHeight="1">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="33" ht="35" customHeight="1">
       <c r="A33" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" ht="35" customHeight="1">
@@ -1541,16 +1627,16 @@
         <v>13</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" ht="63" customHeight="1">
@@ -1558,232 +1644,250 @@
         <v>14</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="36" ht="21" customHeight="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="36" ht="35" customHeight="1">
       <c r="A36" s="12" t="s">
         <v>15</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="37" ht="21" customHeight="1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" ht="63" customHeight="1">
       <c r="A37" s="12" t="s">
         <v>16</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="38" ht="35" customHeight="1">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="38" ht="21" customHeight="1">
       <c r="A38" s="12" t="s">
         <v>17</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E38" s="13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="39" ht="21" customHeight="1">
+      <c r="A39" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D39" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" ht="35" customHeight="1">
+      <c r="A40" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E40" s="13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" ht="35" customHeight="1">
+      <c r="A41" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D41" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="E41" s="13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="39" ht="16" customHeight="1"/>
-    <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="B40" s="9"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-    </row>
-    <row r="41" ht="6" customHeight="1"/>
-    <row r="42" ht="21" customHeight="1">
-      <c r="A42" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="43" ht="35" customHeight="1">
-      <c r="A43" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="D43" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="44" ht="35" customHeight="1">
-      <c r="A44" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B44" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="C44" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="D44" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="E44" s="11" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="45" ht="35" customHeight="1">
-      <c r="A45" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B45" s="11" t="s">
+    <row r="42" ht="16" customHeight="1"/>
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C45" s="11" t="s">
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+    </row>
+    <row r="44" ht="6" customHeight="1"/>
+    <row r="45" ht="21" customHeight="1">
+      <c r="A45" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="D45" s="11" t="s">
+      <c r="B45" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="E45" s="11" t="s">
+      <c r="C45" s="10" t="s">
         <v>130</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="46" ht="35" customHeight="1">
       <c r="A46" s="12" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47" ht="35" customHeight="1">
       <c r="A47" s="12" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="48" ht="16" customHeight="1"/>
-    <row r="49" ht="24" customHeight="1">
-      <c r="A49" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-    </row>
-    <row r="50" ht="6" customHeight="1"/>
-    <row r="51" ht="35" customHeight="1">
-      <c r="A51" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="B51" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="C51" s="11"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-    </row>
-    <row r="52" ht="35" customHeight="1">
-      <c r="A52" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="B52" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="C52" s="11"/>
-      <c r="D52" s="11"/>
-      <c r="E52" s="11"/>
-    </row>
-    <row r="53" ht="35" customHeight="1">
-      <c r="A53" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="B53" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-    </row>
-    <row r="54" ht="21" customHeight="1">
+    </row>
+    <row r="48" ht="35" customHeight="1">
+      <c r="A48" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C48" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D48" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="E48" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="49" ht="35" customHeight="1">
+      <c r="A49" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C49" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E49" s="11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="50" ht="35" customHeight="1">
+      <c r="A50" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="51" ht="16" customHeight="1"/>
+    <row r="52" ht="24" customHeight="1">
+      <c r="A52" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+    </row>
+    <row r="53" ht="6" customHeight="1"/>
+    <row r="54" ht="35" customHeight="1">
       <c r="A54" s="12" t="s">
-        <v>15</v>
+        <v>149</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="C54" s="11"/>
       <c r="D54" s="11"/>
@@ -1791,10 +1895,10 @@
     </row>
     <row r="55" ht="35" customHeight="1">
       <c r="A55" s="12" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="C55" s="11"/>
       <c r="D55" s="11"/>
@@ -1802,21 +1906,21 @@
     </row>
     <row r="56" ht="35" customHeight="1">
       <c r="A56" s="12" t="s">
-        <v>143</v>
+        <v>7</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C56" s="11"/>
       <c r="D56" s="11"/>
       <c r="E56" s="11"/>
     </row>
-    <row r="57" ht="35" customHeight="1">
+    <row r="57" ht="21" customHeight="1">
       <c r="A57" s="12" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C57" s="11"/>
       <c r="D57" s="11"/>
@@ -1824,87 +1928,87 @@
     </row>
     <row r="58" ht="35" customHeight="1">
       <c r="A58" s="12" t="s">
-        <v>0</v>
+        <v>154</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="C58" s="11"/>
       <c r="D58" s="11"/>
       <c r="E58" s="11"/>
     </row>
-    <row r="59" ht="21" customHeight="1">
+    <row r="59" ht="35" customHeight="1">
       <c r="A59" s="12" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="C59" s="11"/>
       <c r="D59" s="11"/>
       <c r="E59" s="11"/>
     </row>
-    <row r="60" ht="16" customHeight="1"/>
-    <row r="61" ht="24" customHeight="1">
-      <c r="A61" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-    </row>
-    <row r="62" ht="6" customHeight="1"/>
-    <row r="63" ht="21" customHeight="1">
-      <c r="A63" s="12" t="s">
+    <row r="60" ht="35" customHeight="1">
+      <c r="A60" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C60" s="11"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="11"/>
+    </row>
+    <row r="61" ht="35" customHeight="1">
+      <c r="A61" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C61" s="11"/>
+      <c r="D61" s="11"/>
+      <c r="E61" s="11"/>
+    </row>
+    <row r="62" ht="21" customHeight="1">
+      <c r="A62" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C62" s="11"/>
+      <c r="D62" s="11"/>
+      <c r="E62" s="11"/>
+    </row>
+    <row r="63" ht="16" customHeight="1"/>
+    <row r="64" ht="24" customHeight="1">
+      <c r="A64" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B64" s="9"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="9"/>
+    </row>
+    <row r="65" ht="6" customHeight="1"/>
+    <row r="66" ht="21" customHeight="1">
+      <c r="A66" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B63" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="C63" s="11"/>
-      <c r="D63" s="11"/>
-      <c r="E63" s="11"/>
-    </row>
-    <row r="64" ht="21" customHeight="1">
-      <c r="A64" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B64" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="C64" s="11"/>
-      <c r="D64" s="11"/>
-      <c r="E64" s="11"/>
-    </row>
-    <row r="65" ht="21" customHeight="1">
-      <c r="A65" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="B65" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="C65" s="11"/>
-      <c r="D65" s="11"/>
-      <c r="E65" s="11"/>
-    </row>
-    <row r="66" ht="35" customHeight="1">
-      <c r="A66" s="12" t="s">
-        <v>154</v>
-      </c>
       <c r="B66" s="11" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
       <c r="E66" s="11"/>
     </row>
-    <row r="67" ht="35" customHeight="1">
+    <row r="67" ht="21" customHeight="1">
       <c r="A67" s="12" t="s">
-        <v>156</v>
+        <v>2</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C67" s="11"/>
       <c r="D67" s="11"/>
@@ -1912,160 +2016,193 @@
     </row>
     <row r="68" ht="21" customHeight="1">
       <c r="A68" s="12" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C68" s="11"/>
       <c r="D68" s="11"/>
       <c r="E68" s="11"/>
     </row>
-    <row r="69" ht="16" customHeight="1"/>
-    <row r="70" ht="24" customHeight="1">
-      <c r="A70" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="B70" s="9"/>
-      <c r="C70" s="9"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="9"/>
-    </row>
-    <row r="71" ht="6" customHeight="1"/>
-    <row r="72" ht="21" customHeight="1">
-      <c r="A72" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="B72" s="10"/>
-      <c r="C72" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="D72" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="E72" s="10"/>
-    </row>
-    <row r="73" ht="21" customHeight="1">
-      <c r="A73" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="B73" s="12"/>
-      <c r="C73" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="D73" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="E73" s="11"/>
-    </row>
-    <row r="74" ht="35" customHeight="1">
-      <c r="A74" s="12" t="s">
+    <row r="69" ht="35" customHeight="1">
+      <c r="A69" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="B74" s="12"/>
-      <c r="C74" s="11" t="s">
+      <c r="B69" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="D74" s="11" t="s">
+      <c r="C69" s="11"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="11"/>
+    </row>
+    <row r="70" ht="35" customHeight="1">
+      <c r="A70" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="E74" s="11"/>
-    </row>
-    <row r="75" ht="35" customHeight="1">
-      <c r="A75" s="12" t="s">
+      <c r="B70" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="B75" s="12"/>
-      <c r="C75" s="11" t="s">
+      <c r="C70" s="11"/>
+      <c r="D70" s="11"/>
+      <c r="E70" s="11"/>
+    </row>
+    <row r="71" ht="21" customHeight="1">
+      <c r="A71" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="D75" s="11" t="s">
+      <c r="B71" s="11" t="s">
         <v>172</v>
       </c>
-      <c r="E75" s="11"/>
-    </row>
-    <row r="76" ht="35" customHeight="1">
+      <c r="C71" s="11"/>
+      <c r="D71" s="11"/>
+      <c r="E71" s="11"/>
+    </row>
+    <row r="72" ht="16" customHeight="1"/>
+    <row r="73" ht="24" customHeight="1">
+      <c r="A73" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B73" s="9"/>
+      <c r="C73" s="9"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="9"/>
+    </row>
+    <row r="74" ht="6" customHeight="1"/>
+    <row r="75" ht="21" customHeight="1">
+      <c r="A75" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="D75" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="E75" s="10"/>
+    </row>
+    <row r="76" ht="21" customHeight="1">
       <c r="A76" s="12" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B76" s="12"/>
       <c r="C76" s="11" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E76" s="11"/>
     </row>
     <row r="77" ht="35" customHeight="1">
       <c r="A77" s="12" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B77" s="12"/>
       <c r="C77" s="11" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D77" s="11" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E77" s="11"/>
     </row>
-    <row r="78" ht="21" customHeight="1">
+    <row r="78" ht="35" customHeight="1">
       <c r="A78" s="12" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B78" s="12"/>
       <c r="C78" s="11" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D78" s="11" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="E78" s="11"/>
     </row>
-    <row r="79" ht="49" customHeight="1">
+    <row r="79" ht="35" customHeight="1">
       <c r="A79" s="12" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B79" s="12"/>
       <c r="C79" s="11" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D79" s="11" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E79" s="11"/>
     </row>
     <row r="80" ht="35" customHeight="1">
       <c r="A80" s="12" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B80" s="12"/>
       <c r="C80" s="11" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="E80" s="11"/>
     </row>
-    <row r="81" ht="35" customHeight="1">
+    <row r="81" ht="21" customHeight="1">
       <c r="A81" s="12" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B81" s="12"/>
       <c r="C81" s="11" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E81" s="11"/>
     </row>
-    <row r="82" ht="18" customHeight="1"/>
-    <row r="83" ht="16" customHeight="1">
-      <c r="A83" s="15" t="s">
-        <v>191</v>
+    <row r="82" ht="49" customHeight="1">
+      <c r="A82" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="B82" s="12"/>
+      <c r="C82" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="D82" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="E82" s="11"/>
+    </row>
+    <row r="83" ht="35" customHeight="1">
+      <c r="A83" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="B83" s="12"/>
+      <c r="C83" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="D83" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="E83" s="11"/>
+    </row>
+    <row r="84" ht="35" customHeight="1">
+      <c r="A84" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="B84" s="12"/>
+      <c r="C84" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="D84" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="E84" s="11"/>
+    </row>
+    <row r="85" ht="18" customHeight="1"/>
+    <row r="86" ht="16" customHeight="1">
+      <c r="A86" s="15" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -2076,27 +2213,21 @@
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="B52:E52"/>
-    <mergeCell ref="B53:E53"/>
     <mergeCell ref="B54:E54"/>
     <mergeCell ref="B55:E55"/>
     <mergeCell ref="B56:E56"/>
     <mergeCell ref="B57:E57"/>
     <mergeCell ref="B58:E58"/>
     <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:E62"/>
     <mergeCell ref="B66:E66"/>
     <mergeCell ref="B67:E67"/>
     <mergeCell ref="B68:E68"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B71:E71"/>
     <mergeCell ref="A75:B75"/>
     <mergeCell ref="D75:E75"/>
     <mergeCell ref="A76:B76"/>
@@ -2111,6 +2242,12 @@
     <mergeCell ref="D80:E80"/>
     <mergeCell ref="A81:B81"/>
     <mergeCell ref="D81:E81"/>
+    <mergeCell ref="A82:B82"/>
+    <mergeCell ref="D82:E82"/>
+    <mergeCell ref="A83:B83"/>
+    <mergeCell ref="D83:E83"/>
+    <mergeCell ref="A84:B84"/>
+    <mergeCell ref="D84:E84"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>